<commit_message>
Update REST API documentation
</commit_message>
<xml_diff>
--- a/RestAPI/developer_feedback/schema_update_requests.xlsx
+++ b/RestAPI/developer_feedback/schema_update_requests.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,8 +48,13 @@
       <color rgb="007F6000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00006100"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -74,6 +79,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -103,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -121,6 +131,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -488,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -516,6 +529,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -598,14 +612,14 @@
           <t>HTTPS, FTPS, SFTP</t>
         </is>
       </c>
-      <c r="H5" s="6" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Source list read 'FTPS, HTTPS, FTPS' (FTPS listed twice); the duplicate was read as SFTP per the review call. Please confirm the exact set.</t>
+          <t>Done 2026-07-16 - dev added transfer_protocol enum; integrated both channels.</t>
         </is>
       </c>
     </row>
@@ -645,14 +659,14 @@
 Also: File-based update, USB update</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>Server-based methods apply to the URL download. File-based and USB updates are separate mechanisms that do not use this API.</t>
+          <t>Done 2026-07-16 - dev added transfer_protocol + USB; integrated both channels.</t>
         </is>
       </c>
     </row>
@@ -690,14 +704,14 @@
           <t>Operations: Add (install), List, Delete</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>Current coverage: MQTT has set_installCACertificate (add) and del_CACertificate (delete); no list operation. REST has none. Please add the missing operations to complete CRUD on both channels.</t>
+          <t>Done 2026-07-16 - CA add/list/delete integrated; MQTT list op created + install/delete un-excluded.</t>
         </is>
       </c>
     </row>
@@ -736,14 +750,14 @@
           <t>Move from: Network -&gt; System</t>
         </is>
       </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>Currently tagged 'Network' in REST (getHostName / setHostName) and 'network' in MQTT (get_hostname / set_hostname). A System tag already exists in both specs.</t>
+          <t>Done 2026-07-16 - hostName retagged to System on both channels.</t>
         </is>
       </c>
     </row>
@@ -782,14 +796,14 @@
           <t>Payloads: Install, Delete</t>
         </is>
       </c>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Currently only get/set eSimConfig exist on both channels. Please add the install and delete payloads to the schema.</t>
+          <t>Done 2026-07-16 - eSim add/delete via operation enum + activationID; both channels.</t>
         </is>
       </c>
     </row>

</xml_diff>